<commit_message>
Added three class and related changes for wuxi audits
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/AVS_CQV_TestData.xlsx
+++ b/src/test/resources/TestData/AVS_CQV_TestData.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kaveri.Bedar\git\AVS-QUAL-FLOW\src\test\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14CA9E4A-5162-4615-8BC9-97A628AC4580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11D34D45-C747-4C4E-ABFE-F17BD83349A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CQV" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>AssetName</t>
   </si>
@@ -44,9 +43,6 @@
   </si>
   <si>
     <t>Amphenol</t>
-  </si>
-  <si>
-    <t>10.17.18.94</t>
   </si>
   <si>
     <t>AVS_Caliberation</t>
@@ -432,34 +428,16 @@
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>9</v>
       </c>
       <c r="E2" s="2">
         <v>46</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{074AFF5F-76E6-4981-97A0-D1B7A899F69F}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="10.7265625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>